<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.002-06 Les lanternes de Chouchou
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.002-06.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.002-06.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>perron au crépuscule</t>
+          <t>perron au crépuscule, pots de confiture, sucre, papier jaune, pierre tiède, fenêtre jaune</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chouchou, Mila, papa</t>
+          <t>Chouchou, Mila, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut des lanternes de papier dans deux pots. Mila arrive. Un rire commence. Papa dit : le corps n'est pas une blague. Un couvercle résiste. Ils les lèvent vers le dernier soleil.</t>
+          <t>Un reste de sucre capte le dernier soleil, au fond des pots. Sur la pierre, un éclat de perron brille. Chouchou veut des lanternes maintenant. Elle pousse trop vite : le papier se froisse, le couvercle résiste, l'éclat glisse. Mila prend son temps. Un petit rire commence, puis s'arrête. Elle refuse de foncer, propose. Mila regarde. Merci vécu. Lever trop vite : le papier file. Elle refuse, retrouve l'éclat. L'éclat de perron tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La pierre du perron garde la chaleur du jour. Deux pots de confiture attendent, vides. Un reste de sucre brille au fond. Un grillon commence, tout près. La fenêtre de la cuisine est jaune. Une casserole cliquette, très loin. Ça sent l'herbe coupée. Un papillon de nuit tourne. Le ciel devient un peu violet. Tu as senti la pierre, Chouchou ? Elle est encore chaude. Oui. Le soleil l'a gardée. En ce moment, Chouchou prend un pot. Le verre est lisse et un peu froid. Un reste d'étiquette colle encore. Je veux des lanternes. Avec du papier jaune. On les lève vers le ciel ? Oui. Mila arrive sur la première marche. Ses chaussons font un bruit mou. Mila n'a pas la même forme. Les corps sont différents. Un petit rire commence. Le corps n'est pas une blague. On joue. Chouchou ferme la bouche. Mila, tu veux une lanterne ? Oui. Papa tend deux papiers jaunes. Ils froissent un peu. Le jaune est fin comme une peau d'oignon. Il fait un bruit de papier. Le mien aussi.</t>
+          <t>Un reste de sucre capte le dernier soleil. Il brille au fond d'un pot de confiture. Ça brille, papa ! Tu le vois, dans le verre ? Oui, un petit point. Deux pots vides attendent au bord du perron. Le verre est lisse, un peu froid. Le perron est tiède, sous tes pieds ? Oui, maman. La pierre est chaude. Sur la pierre, un éclat de perron brille. Il brille aussi. C'est le soleil, sur la pierre ? Oui, tout petit. Le ciel devient violet, au-dessus du toit. Ça sent l'herbe coupée, près des marches. Ça sent le sucre aussi. Un peu, oui. Un papillon de nuit tourne près de la fenêtre. La fenêtre de la cuisine est jaune. Je veux des lanternes, maintenant ! Avec les pots ? Oui, et du papier jaune. On les lève vers le ciel ? Oui, maman ! Papa tend deux papiers jaunes. Ils froissent, fins, entre les doigts. Il fait un bruit de papier. En ce moment, Chouchou pousse le papier trop vite. Le papier se froisse au fond du pot. Le sucre colle au jaune. Oh. Le couvercle reste coincé. Il ne veut pas ! Mila arrive sur la première marche. Ses chaussons font un bruit mou. Elle prend son temps, un pied, puis l'autre. Mila ! J'arrive. Tes chaussons sont mous, Mila ? Oui. Les lanternes, maintenant, Mila ! Chouchou tire le pot trop vite vers Mila. Non. Mila recule d'une marche. Oh. Un petit rire commence, chez Chouchou. Mila baisse les yeux. Ses épaules se serrent un peu. Le rire s'arrête net. Chouchou ferme la bouche. Ses joues sont chaudes, un peu. L'éclat de perron glisse sur la pierre. Il part. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à Mila, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Tes mains tiennent le verre ? Oui, maman. Les mots se perdent près des pots. Personne n'entend la fin. Le papier reste froissé, au fond.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La pierre du perron garde la chaleur du jour. Deux pots de confiture attendent, vides. Un reste de sucre brille au fond. Un grillon commence, tout près. La fenêtre de la cuisine est jaune. Une casserole cliquette, très loin. Ça sent l'herbe coupée. Un papillon de nuit tourne. Le ciel devient un peu violet. Tu as senti la pierre, Chouchou ? Elle est encore chaude. Oui. Le soleil l'a gardée. En ce moment, Chouchou prend un pot. Le verre est lisse et un peu froid. Un reste d'étiquette colle encore. Je veux des lanternes. Avec du papier jaune. On les lève vers le ciel ? Oui. Mila arrive sur la première marche. Ses chaussons font un bruit mou. Mila n'a pas la même forme. Les corps sont différents. Un petit rire commence. Le corps n'est pas une blague. On joue. Chouchou ferme la bouche. Mila, tu veux une lanterne ? Oui. Papa tend deux papiers jaunes. Ils froissent un peu. Le jaune est fin comme une peau d'oignon. Il fait un bruit de papier. Le mien aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un reste de sucre capte le dernier soleil. Il brille au fond d'un pot de confiture. Ça brille, papa ! Tu le vois, dans le verre ? Oui, un petit point. Deux pots vides attendent au bord du perron. Le verre est lisse, un peu froid. Le perron est tiède, sous tes pieds ? Oui, maman. La pierre est chaude. Sur la pierre, un &lt;emphasis level="moderate"&gt;éclat de perron&lt;/emphasis&gt; brille. Il brille aussi. C'est le soleil, sur la pierre ? Oui, tout petit. Le ciel devient violet, au-dessus du toit. Ça sent l'herbe coupée, près des marches. Ça sent le sucre aussi. Un peu, oui. Un papillon de nuit tourne près de la fenêtre. La fenêtre de la cuisine est jaune. Je veux des lanternes, maintenant ! Avec les pots ? Oui, et du papier jaune. On les lève vers le ciel ? Oui, maman ! Papa tend deux papiers jaunes. Ils froissent, fins, entre les doigts. Il fait un bruit de papier. En ce moment, Chouchou pousse le papier trop vite. Le papier se froisse au fond du pot. Le sucre colle au jaune. Oh. Le couvercle reste coincé. Il ne veut pas ! Mila arrive sur la première marche. Ses chaussons font un bruit mou. Elle prend son temps, un pied, puis l'autre. Mila ! J'arrive. Tes chaussons sont mous, Mila ? Oui. Les lanternes, maintenant, Mila ! Chouchou tire le pot trop vite vers Mila. Non. Mila recule d'une marche. Oh. Un petit rire commence, chez Chouchou. Mila baisse les yeux. Ses épaules se serrent un peu. Le rire s'arrête net. Chouchou ferme la bouche. Ses joues sont chaudes, un peu. L'éclat de perron glisse sur la pierre. Il part. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à Mila, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Tes mains tiennent le verre ? Oui, maman. Les mots se perdent près des pots. Personne n'entend la fin. Le papier reste froissé, au fond.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Agathe est dans la cuisine avec papa. Inès arrive. Elles n'ont pas la même forme. Les &lt;emphasis&gt;corps&lt;/emphasis&gt; sont différents. Un petit rire commence. Papa parle tout de suite. Papa dit : le corps n'est pas une blague. On joue. Agathe ferme la bouche. Elle tend un emporte-pièce. La pâte est froide. Elles jouent. Elles font des formes. Parce que le corps n'est pas une blague, l'amitié reste. On ne commente pas le corps pour rabaisser. Agathe et Inès pressent la pâte. Ça sent la farine. Papa sourit. Elles jouent ensemble. Le corps n'est pas une blague. [pause]</t>
+          <t>Un reste de sucre capte le dernier soleil. Il brille au fond d'un pot de confiture. Ça brille, papa ! Tu le vois, dans le verre ? Oui, un petit point. Deux pots vides attendent au bord du perron. Le verre est lisse, un peu froid. Le perron est tiède, sous tes pieds ? Oui, maman. La pierre est chaude. Sur la pierre, un &lt;emphasis&gt;éclat de perron&lt;/emphasis&gt; brille. Il brille aussi. C'est le soleil, sur la pierre ? Oui, tout petit. Le ciel devient violet, au-dessus du toit. Ça sent l'herbe coupée, près des marches. Ça sent le sucre aussi. Un peu, oui. Un papillon de nuit tourne près de la fenêtre. La fenêtre de la cuisine est jaune. Je veux des lanternes, maintenant ! Avec les pots ? Oui, et du papier jaune. On les lève vers le ciel ? Oui, maman ! Papa tend deux papiers jaunes. Ils froissent, fins, entre les doigts. Il fait un bruit de papier. En ce moment, Chouchou pousse le papier trop vite. Le papier se froisse au fond du pot. Le sucre colle au jaune. Oh. Le couvercle reste coincé. Il ne veut pas ! Mila arrive sur la première marche. Ses chaussons font un bruit mou. Elle prend son temps, un pied, puis l'autre. Mila ! J'arrive. Tes chaussons sont mous, Mila ? Oui. Les lanternes, maintenant, Mila ! Chouchou tire le pot trop vite vers Mila. Non. Mila recule d'une marche. Oh. Un petit rire commence, chez Chouchou. Mila baisse les yeux. Ses épaules se serrent un peu. Le rire s'arrête net. Chouchou ferme la bouche. Ses joues sont chaudes, un peu. L'éclat de perron glisse sur la pierre. Il part. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à Mila, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Tes mains tiennent le verre ? Oui, maman. Les mots se perdent près des pots. Personne n'entend la fin. Le papier reste froissé, au fond. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>éclat de perron</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,44 +1321,82 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=elle_veut_les_lanternes_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La pierre du perron garde la chaleur du jour.
-narrateur|Deux pots de confiture attendent, vides.
-narrateur|Un reste de sucre brille au fond.
-narrateur|Un grillon commence, tout près.
+          <t>narrateur|Un reste de sucre capte le dernier soleil.
+narrateur|Il brille au fond d'un pot de confiture.
+enfant-f|Ça brille, papa !
+papa|Tu le vois, dans le verre ?
+enfant-f|Oui, un petit point.
+narrateur|Deux pots vides attendent au bord du perron.
+narrateur|Le verre est lisse, un peu froid.
+maman|Le perron est tiède, sous tes pieds ?
+enfant-f|Oui, maman.
+enfant-f|La pierre est chaude.
+narrateur|Sur la pierre, un éclat de perron brille.
+enfant-f|Il brille aussi.
+papa|C'est le soleil, sur la pierre ?
+enfant-f|Oui, tout petit.
+narrateur|Le ciel devient violet, au-dessus du toit.
+narrateur|Ça sent l'herbe coupée, près des marches.
+enfant-f|Ça sent le sucre aussi.
+maman|Un peu, oui.
+narrateur|Un papillon de nuit tourne près de la fenêtre.
 narrateur|La fenêtre de la cuisine est jaune.
-narrateur|Une casserole cliquette, très loin.
-narrateur|Ça sent l'herbe coupée.
-narrateur|Un papillon de nuit tourne.
-narrateur|Le ciel devient un peu violet.
-papa|Tu as senti la pierre, Chouchou ?
-enfant-m|Elle est encore chaude.
-papa|Oui.
-papa|Le soleil l'a gardée.
-narrateur|En ce moment, Chouchou prend un pot.
-narrateur|Le verre est lisse et un peu froid.
-narrateur|Un reste d'étiquette colle encore.
-enfant-m|Je veux des lanternes.
-enfant-m|Avec du papier jaune.
-papa|On les lève vers le ciel ?
-enfant-m|Oui.
+enfant-f|Je veux des lanternes, maintenant !
+papa|Avec les pots ?
+enfant-f|Oui, et du papier jaune.
+maman|On les lève vers le ciel ?
+enfant-f|Oui, maman !
+narrateur|Papa tend deux papiers jaunes.
+narrateur|Ils froissent, fins, entre les doigts.
+enfant-f|Il fait un bruit de papier.
+narrateur|En ce moment, Chouchou pousse le papier trop vite.
+narrateur|Le papier se froisse au fond du pot.
+narrateur|Le sucre colle au jaune.
+enfant-f|Oh.
+narrateur|Le couvercle reste coincé.
+enfant-f|Il ne veut pas !
 narrateur|Mila arrive sur la première marche.
 narrateur|Ses chaussons font un bruit mou.
-narrateur|Mila n'a pas la même forme.
-narrateur|Les corps sont différents.
-narrateur|Un petit rire commence.
-papa|Le corps n'est pas une blague.
-papa|On joue.
+narrateur|Elle prend son temps, un pied, puis l'autre.
+enfant-f|Mila !
+copine|J'arrive.
+maman|Tes chaussons sont mous, Mila ?
+copine|Oui.
+enfant-f|Les lanternes, maintenant, Mila !
+narrateur|Chouchou tire le pot trop vite vers Mila.
+copine|Non.
+narrateur|Mila recule d'une marche.
+enfant-f|Oh.
+narrateur|Un petit rire commence, chez Chouchou.
+narrateur|Mila baisse les yeux.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Le rire s'arrête net.
 narrateur|Chouchou ferme la bouche.
-enfant-m|Mila, tu veux une lanterne ?
-copine|Oui.
-narrateur|Papa tend deux papiers jaunes.
-narrateur|Ils froissent un peu.
-narrateur|Le jaune est fin comme une peau d'oignon.
-enfant-m|Il fait un bruit de papier.
-copine|Le mien aussi.</t>
+narrateur|Ses joues sont chaudes, un peu.
+narrateur|L'éclat de perron glisse sur la pierre.
+enfant-f|Il part.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Tu parles à Mila, Chouchou ?
+narrateur|Papa s'accroupit à la même hauteur.
+enfant-f|Oui, papa.
+maman|Tes mains tiennent le verre ?
+enfant-f|Oui, maman.
+narrateur|Les mots se perdent près des pots.
+narrateur|Personne n'entend la fin.
+narrateur|Le papier reste froissé, au fond.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>sucre,pots,papier</t>
         </is>
       </c>
     </row>
@@ -1390,12 +1428,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps n'est pas une blague. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le corps n'est pas une &lt;emphasis level="moderate"&gt;blague&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le corps n'est pas une &lt;emphasis&gt;blague&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1420,7 +1458,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On joue. Le corps n'est pas une blague. Que fait-on ?</t>
+          <t>On joue. Que fait Chouchou ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1458,7 +1496,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1469,7 +1507,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1484,38 +1522,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>blague</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1530,17 +1568,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_rire_s_est_arrete_elles_peuvent_jouer; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1573,17 +1611,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou glisse le papier dans son pot. Mila glisse le sien. Un couvercle reste coincé. Il ne veut pas. On tourne ensemble. Ils tiennent le verre. Le couvercle vient, tout à coup. Bravo, Chouchou. Vous avez ouvert. Vous jouez. Le papier jaune s'installe. Il se colle un peu au verre. Ils lèvent les pots. Le dernier soleil traverse le jaune. Ça brille. La mienne aussi. L'amitié ne dépend pas de la forme. On joue. Ils s'assoient sur la pierre chaude. Le grillon recommence. Une fourmi croise le perron. On la laisse passer. Ils restent un moment, tout calmes.</t>
+          <t>Chouchou avance le pot trop vite. Tu pousses le papier, maintenant ! Les mots se bousculent dans sa bouche. Non. Mila reste sur la marche. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le pot, un peu. Le papier est froissé, Chouchou ? Papa reste à sa hauteur. Le sucre colle, sous tes doigts. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Tu veux tourner le couvercle ? Mila ne dit rien. Elle s'assoit sur la marche. Je regarde. D'accord. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens le verre des deux mains ? Oui, maman. Il est froid. Tu parles du sucre, si tu veux ? Le sucre capte le soleil. On reste au perron, Chouchou ? Oui. Chouchou glisse le papier sans presser. Le jaune se pose contre le verre. Mila tourne le couvercle, sans se presser. Le couvercle vient, sans un à-coup. Il est ouvert. Le mien aussi. Tu as entendu le verre ? Oui, papa. Elles lèvent un peu les pots. Le dernier soleil traverse le jaune. Ça brille. La mienne aussi. Le ventre de Chouchou se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou glisse le papier dans son pot. Mila glisse le sien. Un couvercle reste coincé. Il ne veut pas. On tourne ensemble. Ils tiennent le verre. Le couvercle vient, tout à coup. Bravo, Chouchou. Vous avez ouvert. Vous jouez. Le papier jaune s'installe. Il se colle un peu au verre. Ils lèvent les pots. Le dernier soleil traverse le jaune. Ça brille. La mienne aussi. L'amitié ne dépend pas de la forme. On joue. Ils s'assoient sur la pierre chaude. Le grillon recommence. Une fourmi croise le perron. On la laisse passer. Ils restent un moment, tout calmes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou avance le pot trop vite. Tu pousses le &lt;emphasis level="moderate"&gt;papier&lt;/emphasis&gt;, maintenant ! Les mots se bousculent dans sa bouche. Non. Mila reste sur la marche. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le pot, un peu. Le papier est froissé, Chouchou ? Papa reste à sa hauteur. Le sucre colle, sous tes doigts. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Tu veux tourner le couvercle ? Mila ne dit rien. Elle s'assoit sur la marche. Je regarde. D'accord. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens le verre des deux mains ? Oui, maman. Il est froid. Tu parles du sucre, si tu veux ? Le sucre capte le soleil. On reste au perron, Chouchou ? Oui. Chouchou glisse le papier sans presser. Le jaune se pose contre le verre. Mila tourne le couvercle, sans se presser. Le couvercle vient, sans un à-coup. Il est ouvert. Le mien aussi. Tu as entendu le verre ? Oui, papa. Elles lèvent un peu les pots. Le dernier soleil traverse le jaune. Ça brille. La mienne aussi. Le ventre de Chouchou se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Agathe a entendu papa. Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Agathe et Inès ont joué. [pause]</t>
+          <t>Chouchou avance le pot trop vite. Tu pousses le &lt;emphasis&gt;papier&lt;/emphasis&gt;, maintenant ! Les mots se bousculent dans sa bouche. Non. Mila reste sur la marche. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le pot, un peu. Le papier est froissé, Chouchou ? Papa reste à sa hauteur. Le sucre colle, sous tes doigts. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Tu veux tourner le couvercle ? Mila ne dit rien. Elle s'assoit sur la marche. Je regarde. D'accord. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens le verre des deux mains ? Oui, maman. Il est froid. Tu parles du sucre, si tu veux ? Le sucre capte le soleil. On reste au perron, Chouchou ? Oui. Chouchou glisse le papier sans presser. Le jaune se pose contre le verre. Mila tourne le couvercle, sans se presser. Le couvercle vient, sans un à-coup. Il est ouvert. Le mien aussi. Tu as entendu le verre ? Oui, papa. Elles lèvent un peu les pots. Le dernier soleil traverse le jaune. Ça brille. La mienne aussi. Le ventre de Chouchou se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1630,7 +1668,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1638,10 +1676,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1664,30 +1702,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>papier</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1696,10 +1734,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1712,34 +1750,57 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_propose_mila_regarde_elles_glissent_le_papier; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou glisse le papier dans son pot.
-narrateur|Mila glisse le sien.
-narrateur|Un couvercle reste coincé.
-copine|Il ne veut pas.
-enfant-m|On tourne ensemble.
-narrateur|Ils tiennent le verre.
-narrateur|Le couvercle vient, tout à coup.
-papa|Bravo, Chouchou.
-papa|Vous avez ouvert.
-papa|Vous jouez.
-narrateur|Le papier jaune s'installe.
-narrateur|Il se colle un peu au verre.
-narrateur|Ils lèvent les pots.
+          <t>narrateur|Chouchou avance le pot trop vite.
+enfant-f|Tu pousses le papier, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Non.
+narrateur|Mila reste sur la marche.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Chouchou refuse de foncer.
+narrateur|Elle recule le pot, un peu.
+papa|Le papier est froissé, Chouchou ?
+narrateur|Papa reste à sa hauteur.
+maman|Le sucre colle, sous tes doigts.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Chouchou attend que le silence arrive.
+enfant-f|Tu veux tourner le couvercle ?
+narrateur|Mila ne dit rien.
+narrateur|Elle s'assoit sur la marche.
+copine|Je regarde.
+enfant-f|D'accord.
+papa|Merci, Chouchou.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu tiens le verre des deux mains ?
+enfant-f|Oui, maman.
+enfant-f|Il est froid.
+papa|Tu parles du sucre, si tu veux ?
+enfant-f|Le sucre capte le soleil.
+maman|On reste au perron, Chouchou ?
+enfant-f|Oui.
+narrateur|Chouchou glisse le papier sans presser.
+narrateur|Le jaune se pose contre le verre.
+narrateur|Mila tourne le couvercle, sans se presser.
+narrateur|Le couvercle vient, sans un à-coup.
+enfant-f|Il est ouvert.
+copine|Le mien aussi.
+papa|Tu as entendu le verre ?
+enfant-f|Oui, papa.
+narrateur|Elles lèvent un peu les pots.
 narrateur|Le dernier soleil traverse le jaune.
-enfant-m|Ça brille.
+enfant-f|Ça brille.
 copine|La mienne aussi.
-papa|L'amitié ne dépend pas de la forme.
-papa|On joue.
-narrateur|Ils s'assoient sur la pierre chaude.
-narrateur|Le grillon recommence.
-narrateur|Une fourmi croise le perron.
-papa|On la laisse passer.
-narrateur|Ils restent un moment, tout calmes.</t>
+narrateur|Le ventre de Chouchou se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>verre,couvercle</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1827,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On les pose un moment ? Oui. Les deux pots reposent côte à côte. La fenêtre jaune leur fait face. C'est comme deux lunes. Deux petites. Tu as fini de les lever ? Oui, papa. Chouchou essuie le verre. Mila essuie l'autre. Les pots cliquettent un peu. Merci, Mila. Merci, Chouchou. La pierre refroidit un peu. Le ciel est presque bleu nuit.</t>
+          <t>Chouchou veut lever les pots, d'un coup. On les lève, maintenant ! Elle lève trop vite. Le papier glisse vers le bord. Oh. Papa n'a pas fini sa phrase. Le papier file, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le perron, un instant. Elle observe le pot, écoute la pierre. Sur la pierre, un éclat de perron luit. Il est là. Tu lèves le tien, si tu veux ? Plus tard. D'accord. Mila reste à regarder. Chouchou lève le pot sans presser. Le jaune s'allume dans le verre. C'est une lanterne. Tu restes un peu ? Oui, papa. Les pots sont près de la marche. On les pose ? Oui, sur la pierre. Le verre sent le sucre. Il colle aux doigts. Comme le reste, oui. Mila lève le sien, sans un mot. Le jaune s'allume aussi, chez elle. La mienne brille. Les deux brillent.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On les pose un moment ? Oui. Les deux pots reposent côte à côte. La fenêtre jaune leur fait face. C'est comme deux lunes. Deux petites. Tu as fini de les lever ? Oui, papa. Chouchou essuie le verre. Mila essuie l'autre. Les pots cliquettent un peu. Merci, Mila. Merci, Chouchou. La pierre refroidit un peu. Le ciel est presque bleu nuit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou veut lever les pots, d'un coup. On les lève, maintenant ! Elle lève trop vite. Le papier glisse vers le bord. Oh. Papa n'a pas fini sa phrase. Le papier file, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le perron, un instant. Elle observe le pot, écoute la pierre. Sur la pierre, un &lt;emphasis level="moderate"&gt;éclat de perron&lt;/emphasis&gt; luit. Il est là. Tu lèves le tien, si tu veux ? Plus tard. D'accord. Mila reste à regarder. Chouchou lève le pot sans presser. Le jaune s'allume dans le verre. C'est une lanterne. Tu restes un peu ? Oui, papa. Les pots sont près de la marche. On les pose ? Oui, sur la pierre. Le verre sent le sucre. Il colle aux doigts. Comme le reste, oui. Mila lève le sien, sans un mot. Le jaune s'allume aussi, chez elle. La mienne brille. Les deux brillent.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Agathe range un morceau de pâte. Inès range un emporte-pièce. [pause]</t>
+          <t>Chouchou veut lever les pots, d'un coup. On les lève, maintenant ! Elle lève trop vite. Le papier glisse vers le bord. Oh. Papa n'a pas fini sa phrase. Le papier file, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le perron, un instant. Elle observe le pot, écoute la pierre. Sur la pierre, un &lt;emphasis&gt;éclat de perron&lt;/emphasis&gt; luit. Il est là. Tu lèves le tien, si tu veux ? Plus tard. D'accord. Mila reste à regarder. Chouchou lève le pot sans presser. Le jaune s'allume dans le verre. C'est une lanterne. Tu restes un peu ? Oui, papa. Les pots sont près de la marche. On les pose ? Oui, sur la pierre. Le verre sent le sucre. Il colle aux doigts. Comme le reste, oui. Mila lève le sien, sans un mot. Le jaune s'allume aussi, chez elle. La mienne brille. Les deux brillent. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1823,7 +1884,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1831,10 +1892,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1855,28 +1916,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de perron</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1885,10 +1950,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1899,24 +1964,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_lever_trop_vite; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|On les pose un moment ?
-enfant-m|Oui.
-narrateur|Les deux pots reposent côte à côte.
-narrateur|La fenêtre jaune leur fait face.
-copine|C'est comme deux lunes.
-enfant-m|Deux petites.
-papa|Tu as fini de les lever ?
-enfant-m|Oui, papa.
-narrateur|Chouchou essuie le verre.
-narrateur|Mila essuie l'autre.
-narrateur|Les pots cliquettent un peu.
-enfant-m|Merci, Mila.
-copine|Merci, Chouchou.
-narrateur|La pierre refroidit un peu.
-narrateur|Le ciel est presque bleu nuit.</t>
+          <t>narrateur|Chouchou veut lever les pots, d'un coup.
+enfant-f|On les lève, maintenant !
+narrateur|Elle lève trop vite.
+narrateur|Le papier glisse vers le bord.
+enfant-f|Oh.
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le papier file, Chouchou.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle écoute le perron, un instant.
+narrateur|Elle observe le pot, écoute la pierre.
+narrateur|Sur la pierre, un éclat de perron luit.
+enfant-f|Il est là.
+enfant-f|Tu lèves le tien, si tu veux ?
+copine|Plus tard.
+enfant-f|D'accord.
+narrateur|Mila reste à regarder.
+narrateur|Chouchou lève le pot sans presser.
+narrateur|Le jaune s'allume dans le verre.
+enfant-f|C'est une lanterne.
+papa|Tu restes un peu ?
+enfant-f|Oui, papa.
+maman|Les pots sont près de la marche.
+enfant-f|On les pose ?
+papa|Oui, sur la pierre.
+narrateur|Le verre sent le sucre.
+enfant-f|Il colle aux doigts.
+maman|Comme le reste, oui.
+narrateur|Mila lève le sien, sans un mot.
+narrateur|Le jaune s'allume aussi, chez elle.
+copine|La mienne brille.
+enfant-f|Les deux brillent.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>papier,pierre</t>
         </is>
       </c>
     </row>
@@ -1943,17 +2036,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On a fait des lanternes. Elles ont brillé. Vous avez joué. Le grillon reste dans l'herbe.</t>
+          <t>Elles restent près des pots. Maman pose les deux verres côte à côte. Comme deux lunes, papa. Tu les vois, toi ? Oui, sur la pierre. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Les lanternes sont posées, Chouchou. Oui, avec Mila. L'odeur d'herbe reste sur le perron. Il est là, maman. Oui, sur la pierre. Le ciel est presque bleu nuit. Deux petites. Un peu de sucre tient au verre. L'éclat de perron tient sur la pierre.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>On a fait des lanternes. Elles ont brillé. Vous avez joué. Le grillon reste dans l'herbe.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Elles restent près des pots. Maman pose les deux verres côte à côte. Comme deux lunes, papa. Tu les vois, toi ? Oui, sur la pierre. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Les lanternes sont posées, Chouchou. Oui, avec Mila. L'odeur d'herbe reste sur le perron. Il est là, maman. Oui, sur la pierre. Le ciel est presque bleu nuit. Deux petites. Un peu de sucre tient au verre. L'&lt;emphasis level="moderate"&gt;éclat de perron&lt;/emphasis&gt; tient sur la pierre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Elles restent près des pots. Maman pose les deux verres côte à côte. Comme deux lunes, papa. Tu les vois, toi ? Oui, sur la pierre. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Les lanternes sont posées, Chouchou. Oui, avec Mila. L'odeur d'herbe reste sur le perron. Il est là, maman. Oui, sur la pierre. Le ciel est presque bleu nuit. Deux petites. Un peu de sucre tient au verre. L'&lt;emphasis&gt;éclat de perron&lt;/emphasis&gt; tient sur la pierre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2000,7 +2093,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2008,10 +2101,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2020,12 +2113,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2034,17 +2127,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de perron</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2053,11 +2150,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2066,27 +2163,51 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_pierre; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|On a fait des lanternes.
-copine|Elles ont brillé.
-papa|Vous avez joué.
-narrateur|Le grillon reste dans l'herbe.</t>
+          <t>narrateur|Elles restent près des pots.
+narrateur|Maman pose les deux verres côte à côte.
+enfant-f|Comme deux lunes, papa.
+papa|Tu les vois, toi ?
+enfant-f|Oui, sur la pierre.
+maman|On est bien, ici.
+narrateur|Chouchou glisse le doigt, sans se presser.
+enfant-f|On le sent, maman.
+maman|Tu le sens sur tes doigts ?
+enfant-f|Oui, il colle.
+papa|Les lanternes sont posées, Chouchou.
+enfant-f|Oui, avec Mila.
+narrateur|L'odeur d'herbe reste sur le perron.
+enfant-f|Il est là, maman.
+maman|Oui, sur la pierre.
+narrateur|Le ciel est presque bleu nuit.
+copine|Deux petites.
+narrateur|Un peu de sucre tient au verre.
+narrateur|L'éclat de perron tient sur la pierre.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>perron</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2192,6 +2313,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>